<commit_message>
Updated validation for negative test case to ensure test is fully validated
</commit_message>
<xml_diff>
--- a/rules/CORE-000530/negative/01/data/unit-test-coreid-CG0119-negative.xlsx
+++ b/rules/CORE-000530/negative/01/data/unit-test-coreid-CG0119-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -59,8 +59,17 @@
       <name val="Calibri"/>
       <i/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -74,6 +83,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -97,13 +118,15 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -489,7 +512,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -511,9 +534,129 @@
         <v>Error value</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D2" s="2">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>ARM</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>Zanomaline Low Dose (54 mg)</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>ACTARM</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>Not Assigned</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="2">
+        <v>6</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>ARM</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>Zanomaline Low Dose (54 mg)</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="2">
+        <v>6</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>ACTARM</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>Screen Failure</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D6" s="2">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>ARM</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>Zanomaline High Dose (81 mg)</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D7" s="2">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>ACTARM</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>Screen Failure</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -618,203 +761,203 @@
       <c r="G2" s="5" t="str">
         <v>Date/Time of First Study Treatment</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Date/Time of Last Study Treatment</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Date/Time of Informed Consent</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Date/Time of End of Participation</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Date/Time of Death</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Subject Death Flag</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>Study Site Identifier</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>Date/Time of Birth</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Age</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Age Units</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>Sex</v>
       </c>
-      <c r="R2" s="5" t="str">
+      <c r="R2" s="6" t="str">
         <v>Race</v>
       </c>
-      <c r="S2" s="5" t="str">
+      <c r="S2" s="6" t="str">
         <v>Ethnicity</v>
       </c>
-      <c r="T2" s="5" t="str">
+      <c r="T2" s="6" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="U2" s="5" t="str">
+      <c r="U2" s="6" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="V2" s="5" t="str">
+      <c r="V2" s="6" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="W2" s="5" t="str">
+      <c r="W2" s="6" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="X2" s="5" t="str">
+      <c r="X2" s="6" t="str">
         <v>Country</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
+      <c r="A3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="5" t="str">
+      <c r="B3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="5" t="str">
+      <c r="C3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="5" t="str">
+      <c r="D3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="E3" s="5" t="str">
+      <c r="E3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="5" t="str">
+      <c r="F3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="5" t="str">
+      <c r="G3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="H3" s="5" t="str">
+      <c r="H3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="I3" s="5" t="str">
+      <c r="I3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="J3" s="5" t="str">
+      <c r="J3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="K3" s="5" t="str">
+      <c r="K3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="L3" s="5" t="str">
+      <c r="L3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="M3" s="5" t="str">
+      <c r="M3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="N3" s="5" t="str">
+      <c r="N3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="O3" s="5" t="str">
+      <c r="O3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="P3" s="5" t="str">
+      <c r="P3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="Q3" s="5" t="str">
+      <c r="Q3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="R3" s="5" t="str">
+      <c r="R3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="S3" s="5" t="str">
+      <c r="S3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="T3" s="5" t="str">
+      <c r="T3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="U3" s="5" t="str">
+      <c r="U3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="V3" s="5" t="str">
+      <c r="V3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="W3" s="5" t="str">
+      <c r="W3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="X3" s="5" t="str">
+      <c r="X3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
-        <v>50</v>
-      </c>
-      <c r="E4" s="5">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5">
-        <v>50</v>
-      </c>
-      <c r="J4" s="5">
-        <v>50</v>
-      </c>
-      <c r="K4" s="5">
-        <v>50</v>
-      </c>
-      <c r="L4" s="5">
-        <v>50</v>
-      </c>
-      <c r="M4" s="5">
-        <v>50</v>
-      </c>
-      <c r="N4" s="5">
-        <v>50</v>
-      </c>
-      <c r="O4" s="5">
-        <v>50</v>
-      </c>
-      <c r="P4" s="5">
-        <v>50</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>50</v>
-      </c>
-      <c r="R4" s="5">
-        <v>50</v>
-      </c>
-      <c r="S4" s="5">
-        <v>50</v>
-      </c>
-      <c r="T4" s="5">
-        <v>50</v>
-      </c>
-      <c r="U4" s="5">
-        <v>50</v>
-      </c>
-      <c r="V4" s="5">
-        <v>50</v>
-      </c>
-      <c r="W4" s="5">
-        <v>50</v>
-      </c>
-      <c r="X4" s="5">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
+        <v>50</v>
+      </c>
+      <c r="E4" s="6">
+        <v>50</v>
+      </c>
+      <c r="F4" s="6">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6">
+        <v>50</v>
+      </c>
+      <c r="I4" s="6">
+        <v>50</v>
+      </c>
+      <c r="J4" s="6">
+        <v>50</v>
+      </c>
+      <c r="K4" s="6">
+        <v>50</v>
+      </c>
+      <c r="L4" s="6">
+        <v>50</v>
+      </c>
+      <c r="M4" s="6">
+        <v>50</v>
+      </c>
+      <c r="N4" s="6">
+        <v>50</v>
+      </c>
+      <c r="O4" s="6">
+        <v>50</v>
+      </c>
+      <c r="P4" s="6">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="6">
+        <v>50</v>
+      </c>
+      <c r="R4" s="6">
+        <v>50</v>
+      </c>
+      <c r="S4" s="6">
+        <v>50</v>
+      </c>
+      <c r="T4" s="6">
+        <v>50</v>
+      </c>
+      <c r="U4" s="6">
+        <v>50</v>
+      </c>
+      <c r="V4" s="6">
+        <v>50</v>
+      </c>
+      <c r="W4" s="6">
+        <v>50</v>
+      </c>
+      <c r="X4" s="6">
         <v>50</v>
       </c>
     </row>
@@ -879,13 +1022,13 @@
       <c r="T5" s="4" t="str">
         <v>ZANOMALINE_LOW_DOSE_54_mg</v>
       </c>
-      <c r="U5" s="4" t="str">
+      <c r="U5" s="7" t="str">
         <v>Zanomaline Low Dose (54 mg)</v>
       </c>
       <c r="V5" s="4" t="str">
         <v>ACME_LOW_D</v>
       </c>
-      <c r="W5" s="4" t="str">
+      <c r="W5" s="7" t="str">
         <v>Not Assigned</v>
       </c>
       <c r="X5" s="4" t="str">
@@ -953,13 +1096,13 @@
       <c r="T6" s="4" t="str">
         <v>ZANOMALINE_LOW_DOSE_54_mg</v>
       </c>
-      <c r="U6" s="4" t="str">
+      <c r="U6" s="7" t="str">
         <v>Zanomaline Low Dose (54 mg)</v>
       </c>
       <c r="V6" s="4" t="str">
         <v>ACME_LOW_D</v>
       </c>
-      <c r="W6" s="4" t="str">
+      <c r="W6" s="7" t="str">
         <v>Screen Failure</v>
       </c>
       <c r="X6" s="4" t="str">
@@ -1027,13 +1170,13 @@
       <c r="T7" s="4" t="str">
         <v>ZANOMALINE_HIGH_DOSE_81_mg</v>
       </c>
-      <c r="U7" s="4" t="str">
+      <c r="U7" s="7" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
       <c r="V7" s="4" t="str">
         <v>ACME_HIGH_D</v>
       </c>
-      <c r="W7" s="4" t="str">
+      <c r="W7" s="7" t="str">
         <v>Screen Failure</v>
       </c>
       <c r="X7" s="4" t="str">

</xml_diff>